<commit_message>
add H10-backed weekly ceo report
</commit_message>
<xml_diff>
--- a/reports/weekly_conversion/2026-07-25/Mellanni_Weekly_CEO_Overview_2026-07-25.xlsx
+++ b/reports/weekly_conversion/2026-07-25/Mellanni_Weekly_CEO_Overview_2026-07-25.xlsx
@@ -14,7 +14,8 @@
     <sheet name="Products" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Top ASINs" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Promos" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Keywords" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="H10 Keywords" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="SQP Diagnostics" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Summary'!$A$1:$B$10</definedName>
@@ -24,7 +25,8 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Products'!$A$1:$L$31</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Top ASINs'!$A$1:$O$996</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'Promos'!$A$1:$G$25</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'Keywords'!$A$1:$Q$101</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'H10 Keywords'!$A$1:$U$30</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'SQP Diagnostics'!$A$1:$Q$101</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -57139,6 +57141,2051 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:U30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="42" customWidth="1" min="1" max="1"/>
+    <col width="42" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="19" customWidth="1" min="6" max="6"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="15" customWidth="1" min="10" max="10"/>
+    <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="12" max="12"/>
+    <col width="42" customWidth="1" min="13" max="13"/>
+    <col width="21" customWidth="1" min="14" max="14"/>
+    <col width="17" customWidth="1" min="15" max="15"/>
+    <col width="17" customWidth="1" min="16" max="16"/>
+    <col width="25" customWidth="1" min="17" max="17"/>
+    <col width="25" customWidth="1" min="18" max="18"/>
+    <col width="20" customWidth="1" min="19" max="19"/>
+    <col width="26" customWidth="1" min="20" max="20"/>
+    <col width="19" customWidth="1" min="21" max="21"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>keyword</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>h10_asins</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>search_volume</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>organic_rank</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>sponsored_rank</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>cpr</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>iq_score</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>title_density</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>competing_products</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>keyword_sales</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>cpc</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>trend</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>notes</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>search_query_volume</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>total_purchases</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>brand_purchases</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>est_total_keyword_sales</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>est_brand_keyword_sales</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>brand_ctr</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>brand_purchase_per_click</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>opportunity_score</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>king size sheets set</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>B00NLLUMOE, B00NQDGAP2, B00O35DAL4, B016P42ARU, B0822X1VP7</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="n">
+        <v>130261</v>
+      </c>
+      <c r="D2" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="E2" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="F2" t="n">
+        <v>182.45319</v>
+      </c>
+      <c r="G2" t="n">
+        <v>13026.1</v>
+      </c>
+      <c r="H2" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="I2" s="3" t="n">
+        <v>10000</v>
+      </c>
+      <c r="J2" s="3" t="n">
+        <v>2372</v>
+      </c>
+      <c r="K2" t="n">
+        <v>1.72</v>
+      </c>
+      <c r="L2" t="n">
+        <v>44</v>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>match_type=ppc|organic|sponsored|section-sponsored-brand-header|section-sponsored-video; score=89.80</t>
+        </is>
+      </c>
+      <c r="N2" s="3" t="n">
+        <v>65934</v>
+      </c>
+      <c r="O2" s="3" t="n">
+        <v>1618</v>
+      </c>
+      <c r="P2" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="Q2" s="2" t="n">
+        <v>41242.82</v>
+      </c>
+      <c r="R2" s="2" t="n">
+        <v>778.4299999999999</v>
+      </c>
+      <c r="S2" s="4" t="n">
+        <v>0.0063780203606034</v>
+      </c>
+      <c r="T2" s="4" t="n">
+        <v>0.1217948717948717</v>
+      </c>
+      <c r="U2" t="n">
+        <v>83.7</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>twin sheets</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>B00NLLUMOE, B00NQDGAP2, B00O35DAL4, B016P42ARU, B0822X1VP7</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="n">
+        <v>74897</v>
+      </c>
+      <c r="D3" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="E3" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="F3" t="n">
+        <v>115.92751</v>
+      </c>
+      <c r="G3" t="n">
+        <v>3744.85</v>
+      </c>
+      <c r="H3" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="I3" s="3" t="n">
+        <v>20000</v>
+      </c>
+      <c r="J3" s="3" t="n">
+        <v>1792</v>
+      </c>
+      <c r="K3" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="L3" t="n">
+        <v>17</v>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>match_type=ppc|organic|sponsored|section-sponsored-video; score=84.20</t>
+        </is>
+      </c>
+      <c r="N3" s="3" t="n">
+        <v>32646</v>
+      </c>
+      <c r="O3" s="3" t="n">
+        <v>1322</v>
+      </c>
+      <c r="P3" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q3" s="2" t="n">
+        <v>14436.24</v>
+      </c>
+      <c r="R3" s="2" t="n">
+        <v>69.94</v>
+      </c>
+      <c r="S3" s="4" t="n">
+        <v>0.0040710584752035</v>
+      </c>
+      <c r="T3" s="4" t="n">
+        <v>0.0909090909090909</v>
+      </c>
+      <c r="U3" t="n">
+        <v>71.2</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>bed sheets</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>B00NLLUMOE, B00NQDGAP2, B00O35DAL4, B016P42ARU, B0822X1VP7</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="n">
+        <v>109567</v>
+      </c>
+      <c r="D4" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="E4" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="F4" t="n">
+        <v>159.11237</v>
+      </c>
+      <c r="G4" t="n">
+        <v>2739.175</v>
+      </c>
+      <c r="H4" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="I4" s="3" t="n">
+        <v>40000</v>
+      </c>
+      <c r="J4" s="3" t="n">
+        <v>1756</v>
+      </c>
+      <c r="K4" t="n">
+        <v>1.42</v>
+      </c>
+      <c r="L4" t="n">
+        <v>35</v>
+      </c>
+      <c r="M4" t="inlineStr">
+        <is>
+          <t>match_type=organic|sponsored|section-sponsored-video; score=89.11</t>
+        </is>
+      </c>
+      <c r="N4" s="3" t="n">
+        <v>64570</v>
+      </c>
+      <c r="O4" s="3" t="n">
+        <v>478</v>
+      </c>
+      <c r="P4" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q4" s="2" t="n">
+        <v>10152.72</v>
+      </c>
+      <c r="R4" s="2" t="n">
+        <v>258.79</v>
+      </c>
+      <c r="S4" s="4" t="n">
+        <v>0.0049378833149866</v>
+      </c>
+      <c r="T4" s="4" t="n">
+        <v>0.0445859872611464</v>
+      </c>
+      <c r="U4" t="n">
+        <v>67.09999999999999</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>king sheets</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>B00NLLUMOE, B00NQDGAP2, B00O35DAL4, B016P42ARU, B0822X1VP7</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="n">
+        <v>69719</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="F5" t="n">
+        <v>109.44443</v>
+      </c>
+      <c r="G5" t="n">
+        <v>3485.95</v>
+      </c>
+      <c r="H5" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="I5" s="3" t="n">
+        <v>20000</v>
+      </c>
+      <c r="J5" s="3" t="n">
+        <v>1612</v>
+      </c>
+      <c r="K5" t="n">
+        <v>1.89</v>
+      </c>
+      <c r="L5" t="n">
+        <v>72</v>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>match_type=ppc|organic|sponsored|section-sponsored-video|section-sponsored-brand-header; score=85.29</t>
+        </is>
+      </c>
+      <c r="N5" s="3" t="n">
+        <v>28638</v>
+      </c>
+      <c r="O5" s="3" t="n">
+        <v>847</v>
+      </c>
+      <c r="P5" s="3" t="n">
+        <v>37</v>
+      </c>
+      <c r="Q5" s="2" t="n">
+        <v>21590.03</v>
+      </c>
+      <c r="R5" s="2" t="n">
+        <v>1515.89</v>
+      </c>
+      <c r="S5" s="4" t="n">
+        <v>0.0148055751396496</v>
+      </c>
+      <c r="T5" s="4" t="n">
+        <v>0.1355311355311355</v>
+      </c>
+      <c r="U5" t="n">
+        <v>65.8</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>sheets queen size bed set</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>B00NLLUMOE, B00NQDGAP2, B00O35DAL4, B016P42ARU, B0822X1VP7</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="n">
+        <v>59512</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="n">
+        <v>95.6918</v>
+      </c>
+      <c r="G6" t="n">
+        <v>5951.2</v>
+      </c>
+      <c r="H6" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="I6" s="3" t="n">
+        <v>10000</v>
+      </c>
+      <c r="J6" s="3" t="n">
+        <v>1540</v>
+      </c>
+      <c r="K6" t="n">
+        <v>1.67</v>
+      </c>
+      <c r="L6" t="n">
+        <v>42</v>
+      </c>
+      <c r="M6" t="inlineStr">
+        <is>
+          <t>match_type=ppc|organic|sponsored|section-sponsored-video|section-sponsored-brand-header; score=89.63</t>
+        </is>
+      </c>
+      <c r="N6" s="3" t="n">
+        <v>29364</v>
+      </c>
+      <c r="O6" s="3" t="n">
+        <v>648</v>
+      </c>
+      <c r="P6" s="3" t="n">
+        <v>17</v>
+      </c>
+      <c r="Q6" s="2" t="n">
+        <v>13763.52</v>
+      </c>
+      <c r="R6" s="2" t="n">
+        <v>628.49</v>
+      </c>
+      <c r="S6" s="4" t="n">
+        <v>0.0100882173115555</v>
+      </c>
+      <c r="T6" s="4" t="n">
+        <v>0.0735930735930736</v>
+      </c>
+      <c r="U6" t="n">
+        <v>69</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>queen bed sheets</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>B00NLLUMOE, B00NQDGAP2, B00O35DAL4, B016P42ARU, B0822X1VP7</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="n">
+        <v>70938</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F7" t="n">
+        <v>109.28874</v>
+      </c>
+      <c r="G7" t="n">
+        <v>3546.9</v>
+      </c>
+      <c r="H7" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="I7" s="3" t="n">
+        <v>20000</v>
+      </c>
+      <c r="J7" s="3" t="n">
+        <v>1367</v>
+      </c>
+      <c r="K7" t="n">
+        <v>1.61</v>
+      </c>
+      <c r="L7" t="n">
+        <v>9</v>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>match_type=organic|sponsored|section-sponsored-video; score=89.67</t>
+        </is>
+      </c>
+      <c r="N7" s="3" t="n">
+        <v>33686</v>
+      </c>
+      <c r="O7" s="3" t="n">
+        <v>1112</v>
+      </c>
+      <c r="P7" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="Q7" s="2" t="n">
+        <v>23618.88</v>
+      </c>
+      <c r="R7" s="2" t="n">
+        <v>480.61</v>
+      </c>
+      <c r="S7" s="4" t="n">
+        <v>0.0064388673446989</v>
+      </c>
+      <c r="T7" s="4" t="n">
+        <v>0.1477272727272727</v>
+      </c>
+      <c r="U7" t="n">
+        <v>69.3</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>queen size sheets</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>B00NLLUMOE, B00NQDGAP2, B00O35DAL4, B016P42ARU, B0822X1VP7</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>34418</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="F8" t="n">
+        <v>65.50868</v>
+      </c>
+      <c r="G8" t="n">
+        <v>1720.9</v>
+      </c>
+      <c r="H8" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I8" s="3" t="n">
+        <v>20000</v>
+      </c>
+      <c r="J8" s="3" t="n">
+        <v>1357</v>
+      </c>
+      <c r="K8" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="L8" t="n">
+        <v>10</v>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>match_type=organic|sponsored|section-sponsored-video|section-sponsored-brand-header; score=83.21</t>
+        </is>
+      </c>
+      <c r="N8" s="3" t="n">
+        <v>16054</v>
+      </c>
+      <c r="O8" s="3" t="n">
+        <v>593</v>
+      </c>
+      <c r="P8" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q8" s="2" t="n">
+        <v>10668.07</v>
+      </c>
+      <c r="R8" s="2" t="n">
+        <v>184.85</v>
+      </c>
+      <c r="S8" s="4" t="n">
+        <v>0.0059401884473576</v>
+      </c>
+      <c r="T8" s="4" t="n">
+        <v>0.1724137931034483</v>
+      </c>
+      <c r="U8" t="n">
+        <v>54.8</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>cooling sheets</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>B00NLLUMOE, B00NQDGAP2, B00O35DAL4, B016P42ARU, B0822X1VP7</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>84671</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="F9" t="n">
+        <v>131.09243</v>
+      </c>
+      <c r="G9" t="n">
+        <v>2116.775</v>
+      </c>
+      <c r="H9" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="I9" s="3" t="n">
+        <v>40000</v>
+      </c>
+      <c r="J9" s="3" t="n">
+        <v>1356</v>
+      </c>
+      <c r="K9" t="n">
+        <v>1.98</v>
+      </c>
+      <c r="L9" t="n">
+        <v>44</v>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>match_type=organic; score=83.68</t>
+        </is>
+      </c>
+      <c r="N9" s="3" t="n">
+        <v>36897</v>
+      </c>
+      <c r="O9" s="3" t="n">
+        <v>266</v>
+      </c>
+      <c r="P9" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="2" t="n">
+        <v>9041.34</v>
+      </c>
+      <c r="R9" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S9" s="4" t="n">
+        <v>0.009246729815065399</v>
+      </c>
+      <c r="T9" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U9" t="n">
+        <v>55.2</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>queen sheets</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>B00NLLUMOE, B00NQDGAP2, B00O35DAL4, B016P42ARU, B0822X1VP7</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>188972</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F10" t="n">
+        <v>252.31928</v>
+      </c>
+      <c r="G10" t="n">
+        <v>9448.6</v>
+      </c>
+      <c r="H10" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="I10" s="3" t="n">
+        <v>20000</v>
+      </c>
+      <c r="J10" s="3" t="n">
+        <v>1279</v>
+      </c>
+      <c r="K10" t="n">
+        <v>1.59</v>
+      </c>
+      <c r="L10" t="n">
+        <v>73</v>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>match_type=ppc|organic|sponsored|section-sponsored-video; score=93.61</t>
+        </is>
+      </c>
+      <c r="N10" s="3" t="n">
+        <v>74564</v>
+      </c>
+      <c r="O10" s="3" t="n">
+        <v>2564</v>
+      </c>
+      <c r="P10" s="3" t="n">
+        <v>44</v>
+      </c>
+      <c r="Q10" s="2" t="n">
+        <v>51023.6</v>
+      </c>
+      <c r="R10" s="2" t="n">
+        <v>1626.68</v>
+      </c>
+      <c r="S10" s="4" t="n">
+        <v>0.008752158066372501</v>
+      </c>
+      <c r="T10" s="4" t="n">
+        <v>0.1205479452054794</v>
+      </c>
+      <c r="U10" t="n">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>california king sheet sets</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>B00NLLUMOE, B00NQDGAP2, B00O35DAL4, B016P42ARU, B0822X1VP7</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>38359</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="F11" t="n">
+        <v>71.80477</v>
+      </c>
+      <c r="G11" t="n">
+        <v>9589.75</v>
+      </c>
+      <c r="H11" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="I11" s="3" t="n">
+        <v>4000</v>
+      </c>
+      <c r="J11" s="3" t="n">
+        <v>1262</v>
+      </c>
+      <c r="K11" t="n">
+        <v>1.92</v>
+      </c>
+      <c r="L11" t="n">
+        <v>43</v>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>match_type=organic|section-sponsored-brand-header; score=83.67</t>
+        </is>
+      </c>
+      <c r="N11" s="3" t="n">
+        <v>17142</v>
+      </c>
+      <c r="O11" s="3" t="n">
+        <v>514</v>
+      </c>
+      <c r="P11" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q11" s="2" t="n">
+        <v>13358.86</v>
+      </c>
+      <c r="R11" s="2" t="n">
+        <v>44.97</v>
+      </c>
+      <c r="S11" s="4" t="n">
+        <v>0.0092931568572233</v>
+      </c>
+      <c r="T11" s="4" t="n">
+        <v>0.0303030303030303</v>
+      </c>
+      <c r="U11" t="n">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>queen sheet set</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>B00NLLUMOE, B00NQDGAP2, B00O35DAL4, B016P42ARU, B0822X1VP7</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>112569</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F12" t="n">
+        <v>162.36349</v>
+      </c>
+      <c r="G12" t="n">
+        <v>5628.45</v>
+      </c>
+      <c r="H12" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="I12" s="3" t="n">
+        <v>20000</v>
+      </c>
+      <c r="J12" s="3" t="n">
+        <v>1173</v>
+      </c>
+      <c r="K12" t="n">
+        <v>1.68</v>
+      </c>
+      <c r="L12" t="n">
+        <v>12</v>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>match_type=organic|sponsored|section-sponsored-brand-header|section-sponsored-video; score=90.82</t>
+        </is>
+      </c>
+      <c r="N12" s="3" t="n">
+        <v>55981</v>
+      </c>
+      <c r="O12" s="3" t="n">
+        <v>1969</v>
+      </c>
+      <c r="P12" s="3" t="n">
+        <v>25</v>
+      </c>
+      <c r="Q12" s="2" t="n">
+        <v>35422.31</v>
+      </c>
+      <c r="R12" s="2" t="n">
+        <v>924.25</v>
+      </c>
+      <c r="S12" s="4" t="n">
+        <v>0.0077065891337093</v>
+      </c>
+      <c r="T12" s="4" t="n">
+        <v>0.1136363636363636</v>
+      </c>
+      <c r="U12" t="n">
+        <v>61.6</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>bamboo sheets</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>B00NLLUMOE, B00NQDGAP2, B00O35DAL4, B016P42ARU, B0822X1VP7</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>130209</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="F13" t="n">
+        <v>183.03383</v>
+      </c>
+      <c r="G13" t="n">
+        <v>32552.25</v>
+      </c>
+      <c r="H13" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="I13" s="3" t="n">
+        <v>4000</v>
+      </c>
+      <c r="J13" s="3" t="n">
+        <v>1115</v>
+      </c>
+      <c r="K13" t="n">
+        <v>2.95</v>
+      </c>
+      <c r="L13" t="n">
+        <v>40</v>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>match_type=ppc|organic|section-sponsored-brand-header|section-sponsored-video; score=86.78</t>
+        </is>
+      </c>
+      <c r="U13" t="n">
+        <v>68.7</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>cooling sheets queen</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>B00NLLUMOE, B00NQDGAP2, B00O35DAL4, B016P42ARU, B0822X1VP7</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>50097</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="F14" t="n">
+        <v>84.48795000000001</v>
+      </c>
+      <c r="G14" t="n">
+        <v>5009.7</v>
+      </c>
+      <c r="H14" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="I14" s="3" t="n">
+        <v>10000</v>
+      </c>
+      <c r="J14" s="3" t="n">
+        <v>1070</v>
+      </c>
+      <c r="K14" t="n">
+        <v>2.22</v>
+      </c>
+      <c r="L14" t="n">
+        <v>31</v>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t>match_type=organic|section-sponsored-brand-header; score=81.30</t>
+        </is>
+      </c>
+      <c r="N14" s="3" t="n">
+        <v>18433</v>
+      </c>
+      <c r="O14" s="3" t="n">
+        <v>336</v>
+      </c>
+      <c r="P14" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="2" t="n">
+        <v>9404.639999999999</v>
+      </c>
+      <c r="R14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S14" s="4" t="n">
+        <v>0.0135004821600771</v>
+      </c>
+      <c r="T14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U14" t="n">
+        <v>55.7</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>bed sheets queen size</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>B00NLLUMOE, B00NQDGAP2, B00O35DAL4, B016P42ARU, B0822X1VP7</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>45406</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>27</v>
+      </c>
+      <c r="F15" t="n">
+        <v>78.5844</v>
+      </c>
+      <c r="G15" t="n">
+        <v>2270.3</v>
+      </c>
+      <c r="H15" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I15" s="3" t="n">
+        <v>20000</v>
+      </c>
+      <c r="J15" s="3" t="n">
+        <v>1042</v>
+      </c>
+      <c r="K15" t="n">
+        <v>1.76</v>
+      </c>
+      <c r="L15" t="n">
+        <v>43</v>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t>match_type=ppc|organic|section-sponsored-brand-header|section-sponsored-video; score=81.06</t>
+        </is>
+      </c>
+      <c r="N15" s="3" t="n">
+        <v>22537</v>
+      </c>
+      <c r="O15" s="3" t="n">
+        <v>551</v>
+      </c>
+      <c r="P15" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q15" s="2" t="n">
+        <v>11703.24</v>
+      </c>
+      <c r="R15" s="2" t="n">
+        <v>110.91</v>
+      </c>
+      <c r="S15" s="4" t="n">
+        <v>0.005789224952741</v>
+      </c>
+      <c r="T15" s="4" t="n">
+        <v>0.0612244897959183</v>
+      </c>
+      <c r="U15" t="n">
+        <v>49.1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>sheets</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>B00NLLUMOE, B00NQDGAP2, B00O35DAL4, B016P42ARU, B0822X1VP7</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>98465</v>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F16" t="n">
+        <v>153.28997</v>
+      </c>
+      <c r="G16" t="n">
+        <v>984.65</v>
+      </c>
+      <c r="H16" s="3" t="n">
+        <v>37</v>
+      </c>
+      <c r="I16" s="3" t="n">
+        <v>100000</v>
+      </c>
+      <c r="J16" s="3" t="n">
+        <v>997</v>
+      </c>
+      <c r="K16" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="L16" t="n">
+        <v>79</v>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t>match_type=organic|sponsored|section-sponsored-video; score=87.75</t>
+        </is>
+      </c>
+      <c r="N16" s="3" t="n">
+        <v>59978</v>
+      </c>
+      <c r="O16" s="3" t="n">
+        <v>528</v>
+      </c>
+      <c r="P16" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="Q16" s="2" t="n">
+        <v>11214.72</v>
+      </c>
+      <c r="R16" s="2" t="n">
+        <v>665.46</v>
+      </c>
+      <c r="S16" s="4" t="n">
+        <v>0.009040673974091799</v>
+      </c>
+      <c r="T16" s="4" t="n">
+        <v>0.0360721442885771</v>
+      </c>
+      <c r="U16" t="n">
+        <v>42.8</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>king sheet set</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>B00NLLUMOE, B00NQDGAP2, B00O35DAL4, B016P42ARU, B0822X1VP7</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="n">
+        <v>27090</v>
+      </c>
+      <c r="D17" s="3" t="n">
+        <v>15</v>
+      </c>
+      <c r="E17" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="F17" t="n">
+        <v>59.35844</v>
+      </c>
+      <c r="G17" t="n">
+        <v>2709</v>
+      </c>
+      <c r="H17" s="3" t="n">
+        <v>9</v>
+      </c>
+      <c r="I17" s="3" t="n">
+        <v>10000</v>
+      </c>
+      <c r="J17" s="3" t="n">
+        <v>992</v>
+      </c>
+      <c r="K17" t="n">
+        <v>1.94</v>
+      </c>
+      <c r="L17" t="n">
+        <v>32</v>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t>match_type=ppc|organic|sponsored|section-sponsored-video|section-sponsored-brand-header; score=80.10</t>
+        </is>
+      </c>
+      <c r="N17" s="3" t="n">
+        <v>13291</v>
+      </c>
+      <c r="O17" s="3" t="n">
+        <v>423</v>
+      </c>
+      <c r="P17" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q17" s="2" t="n">
+        <v>9775.530000000001</v>
+      </c>
+      <c r="R17" s="2" t="n">
+        <v>286.79</v>
+      </c>
+      <c r="S17" s="4" t="n">
+        <v>0.0094584286803966</v>
+      </c>
+      <c r="T17" s="4" t="n">
+        <v>0.1129032258064516</v>
+      </c>
+      <c r="U17" t="n">
+        <v>33.4</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>full size sheets</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>B00NLLUMOE, B00NQDGAP2, B00O35DAL4, B016P42ARU, B0822X1VP7</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="n">
+        <v>84575</v>
+      </c>
+      <c r="D18" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="F18" t="n">
+        <v>125.51677</v>
+      </c>
+      <c r="G18" t="n">
+        <v>8457.5</v>
+      </c>
+      <c r="H18" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="I18" s="3" t="n">
+        <v>10000</v>
+      </c>
+      <c r="J18" s="3" t="n">
+        <v>981</v>
+      </c>
+      <c r="K18" t="n">
+        <v>1.35</v>
+      </c>
+      <c r="L18" t="n">
+        <v>29</v>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>match_type=ppc|organic|sponsored|section-sponsored-video; score=87.19</t>
+        </is>
+      </c>
+      <c r="N18" s="3" t="n">
+        <v>39272</v>
+      </c>
+      <c r="O18" s="3" t="n">
+        <v>1016</v>
+      </c>
+      <c r="P18" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="Q18" s="2" t="n">
+        <v>15534.64</v>
+      </c>
+      <c r="R18" s="2" t="n">
+        <v>215.82</v>
+      </c>
+      <c r="S18" s="4" t="n">
+        <v>0.0071302614429195</v>
+      </c>
+      <c r="T18" s="4" t="n">
+        <v>0.06451612903225799</v>
+      </c>
+      <c r="U18" t="n">
+        <v>61.4</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>twin xl sheets</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>B00NLLUMOE, B00NQDGAP2, B00O35DAL4, B016P42ARU, B0822X1VP7</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="n">
+        <v>156894</v>
+      </c>
+      <c r="D19" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="F19" t="n">
+        <v>213.50394</v>
+      </c>
+      <c r="G19" t="n">
+        <v>26149</v>
+      </c>
+      <c r="H19" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="I19" s="3" t="n">
+        <v>6000</v>
+      </c>
+      <c r="J19" s="3" t="n">
+        <v>977</v>
+      </c>
+      <c r="K19" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="L19" t="n">
+        <v>91</v>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t>match_type=ppc|organic|section-sponsored-video; score=87.75</t>
+        </is>
+      </c>
+      <c r="N19" s="3" t="n">
+        <v>69302</v>
+      </c>
+      <c r="O19" s="3" t="n">
+        <v>1631</v>
+      </c>
+      <c r="P19" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q19" s="2" t="n">
+        <v>31869.74</v>
+      </c>
+      <c r="R19" s="2" t="n">
+        <v>174.85</v>
+      </c>
+      <c r="S19" s="4" t="n">
+        <v>0.004069672798307</v>
+      </c>
+      <c r="T19" s="4" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="U19" t="n">
+        <v>64.3</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>king size sheets</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>B00NLLUMOE, B00NQDGAP2, B00O35DAL4, B016P42ARU, B0822X1VP7</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="n">
+        <v>29177</v>
+      </c>
+      <c r="D20" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F20" t="n">
+        <v>62.80575</v>
+      </c>
+      <c r="G20" t="n">
+        <v>1458.85</v>
+      </c>
+      <c r="H20" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="I20" s="3" t="n">
+        <v>20000</v>
+      </c>
+      <c r="J20" s="3" t="n">
+        <v>962</v>
+      </c>
+      <c r="K20" t="n">
+        <v>2.03</v>
+      </c>
+      <c r="L20" t="n">
+        <v>12</v>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t>match_type=organic|sponsored|section-sponsored-brand-header|section-sponsored-video; score=82.82</t>
+        </is>
+      </c>
+      <c r="N20" s="3" t="n">
+        <v>14101</v>
+      </c>
+      <c r="O20" s="3" t="n">
+        <v>383</v>
+      </c>
+      <c r="P20" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="Q20" s="2" t="n">
+        <v>9571.17</v>
+      </c>
+      <c r="R20" s="2" t="n">
+        <v>286.79</v>
+      </c>
+      <c r="S20" s="4" t="n">
+        <v>0.007078313253012</v>
+      </c>
+      <c r="T20" s="4" t="n">
+        <v>0.1489361702127659</v>
+      </c>
+      <c r="U20" t="n">
+        <v>24.2</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>full sheet set</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>B00NLLUMOE, B00NQDGAP2, B00O35DAL4, B016P42ARU, B0822X1VP7</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="n">
+        <v>22007</v>
+      </c>
+      <c r="D21" s="3" t="n">
+        <v>13</v>
+      </c>
+      <c r="E21" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="F21" t="n">
+        <v>52.02463</v>
+      </c>
+      <c r="G21" t="n">
+        <v>733.5666666666667</v>
+      </c>
+      <c r="H21" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="I21" s="3" t="n">
+        <v>30000</v>
+      </c>
+      <c r="J21" s="3" t="n">
+        <v>890</v>
+      </c>
+      <c r="K21" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="L21" t="n">
+        <v>43</v>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t>match_type=ppc|organic|sponsored|section-sponsored-video|section-sponsored-brand-header; score=80.36</t>
+        </is>
+      </c>
+      <c r="N21" s="3" t="n">
+        <v>9632</v>
+      </c>
+      <c r="O21" s="3" t="n">
+        <v>284</v>
+      </c>
+      <c r="P21" s="3" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q21" s="2" t="n">
+        <v>4245.8</v>
+      </c>
+      <c r="R21" s="2" t="n">
+        <v>179.85</v>
+      </c>
+      <c r="S21" s="4" t="n">
+        <v>0.0073093638877913</v>
+      </c>
+      <c r="T21" s="4" t="n">
+        <v>0.1351351351351351</v>
+      </c>
+      <c r="U21" t="n">
+        <v>24.3</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>silk sheets</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>B00NLLUMOE, B00NQDGAP2, B00O35DAL4, B016P42ARU, B0822X1VP7</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="n">
+        <v>66098</v>
+      </c>
+      <c r="D22" s="3" t="n">
+        <v>94</v>
+      </c>
+      <c r="F22" t="n">
+        <v>103.52914</v>
+      </c>
+      <c r="G22" t="n">
+        <v>13219.6</v>
+      </c>
+      <c r="H22" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="I22" s="3" t="n">
+        <v>5000</v>
+      </c>
+      <c r="J22" s="3" t="n">
+        <v>860</v>
+      </c>
+      <c r="K22" t="n">
+        <v>1.96</v>
+      </c>
+      <c r="L22" t="n">
+        <v>51</v>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t>match_type=organic|section-sponsored-video; score=81.13</t>
+        </is>
+      </c>
+      <c r="U22" t="n">
+        <v>53.4</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>twin sheets set</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>B00NLLUMOE, B00NQDGAP2, B00O35DAL4, B016P42ARU, B0822X1VP7</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="n">
+        <v>65434</v>
+      </c>
+      <c r="D23" s="3" t="n">
+        <v>19</v>
+      </c>
+      <c r="F23" t="n">
+        <v>104.34528</v>
+      </c>
+      <c r="G23" t="n">
+        <v>6543.400000000001</v>
+      </c>
+      <c r="H23" s="3" t="n">
+        <v>7</v>
+      </c>
+      <c r="I23" s="3" t="n">
+        <v>10000</v>
+      </c>
+      <c r="J23" s="3" t="n">
+        <v>838</v>
+      </c>
+      <c r="K23" t="n">
+        <v>1.27</v>
+      </c>
+      <c r="L23" t="n">
+        <v>31</v>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t>match_type=ppc|organic|section-sponsored-video; score=83.80</t>
+        </is>
+      </c>
+      <c r="N23" s="3" t="n">
+        <v>25872</v>
+      </c>
+      <c r="O23" s="3" t="n">
+        <v>1177</v>
+      </c>
+      <c r="P23" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q23" s="2" t="n">
+        <v>12746.91</v>
+      </c>
+      <c r="R23" s="2" t="n">
+        <v>104.91</v>
+      </c>
+      <c r="S23" s="4" t="n">
+        <v>0.0034425984134111</v>
+      </c>
+      <c r="T23" s="4" t="n">
+        <v>0.1304347826086956</v>
+      </c>
+      <c r="U23" t="n">
+        <v>43.2</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>bamboo sheets queen size</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>B00NLLUMOE, B00NQDGAP2, B00O35DAL4, B016P42ARU, B0822X1VP7</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="n">
+        <v>32857</v>
+      </c>
+      <c r="D24" s="3" t="n">
+        <v>44</v>
+      </c>
+      <c r="F24" t="n">
+        <v>65.89991000000001</v>
+      </c>
+      <c r="G24" t="n">
+        <v>32857</v>
+      </c>
+      <c r="H24" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="I24" s="3" t="n">
+        <v>1000</v>
+      </c>
+      <c r="J24" s="3" t="n">
+        <v>821</v>
+      </c>
+      <c r="K24" t="n">
+        <v>2.64</v>
+      </c>
+      <c r="L24" t="n">
+        <v>32</v>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t>match_type=organic; score=80.44</t>
+        </is>
+      </c>
+      <c r="U24" t="n">
+        <v>39.8</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>queen bedding sets</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>B00NLLUMOE, B00NQDGAP2, B00O35DAL4, B016P42ARU, B0822X1VP7</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="n">
+        <v>50094</v>
+      </c>
+      <c r="D25" s="3" t="n">
+        <v>34</v>
+      </c>
+      <c r="F25" t="n">
+        <v>85.12690000000001</v>
+      </c>
+      <c r="G25" t="n">
+        <v>1669.8</v>
+      </c>
+      <c r="H25" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="I25" s="3" t="n">
+        <v>30000</v>
+      </c>
+      <c r="J25" s="3" t="n">
+        <v>732</v>
+      </c>
+      <c r="K25" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="L25" t="n">
+        <v>58</v>
+      </c>
+      <c r="M25" t="inlineStr">
+        <is>
+          <t>match_type=organic|section-sponsored-brand-header|section-sponsored-video; score=79.96</t>
+        </is>
+      </c>
+      <c r="U25" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>queen sheets deep pocket</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>B00NLLUMOE, B00NQDGAP2, B00O35DAL4, B016P42ARU, B0822X1VP7</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="n">
+        <v>26068</v>
+      </c>
+      <c r="D26" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="E26" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F26" t="n">
+        <v>55.25092000000001</v>
+      </c>
+      <c r="G26" t="n">
+        <v>2606.8</v>
+      </c>
+      <c r="H26" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I26" s="3" t="n">
+        <v>10000</v>
+      </c>
+      <c r="J26" s="3" t="n">
+        <v>671</v>
+      </c>
+      <c r="K26" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="L26" t="n">
+        <v>16</v>
+      </c>
+      <c r="M26" t="inlineStr">
+        <is>
+          <t>match_type=organic|sponsored|section-sponsored-brand-header|section-sponsored-video; score=82.07</t>
+        </is>
+      </c>
+      <c r="N26" s="3" t="n">
+        <v>11186</v>
+      </c>
+      <c r="O26" s="3" t="n">
+        <v>307</v>
+      </c>
+      <c r="P26" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q26" s="2" t="n">
+        <v>6520.679999999999</v>
+      </c>
+      <c r="R26" s="2" t="n">
+        <v>110.91</v>
+      </c>
+      <c r="S26" s="4" t="n">
+        <v>0.0136887608069164</v>
+      </c>
+      <c r="T26" s="4" t="n">
+        <v>0.0526315789473684</v>
+      </c>
+      <c r="U26" t="n">
+        <v>29.1</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>twin bed sheets</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>B00NLLUMOE, B00NQDGAP2, B00O35DAL4, B016P42ARU, B0822X1VP7</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="n">
+        <v>66786</v>
+      </c>
+      <c r="D27" s="3" t="n">
+        <v>53</v>
+      </c>
+      <c r="F27" t="n">
+        <v>104.0266</v>
+      </c>
+      <c r="G27" t="n">
+        <v>6678.6</v>
+      </c>
+      <c r="H27" s="3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I27" s="3" t="n">
+        <v>10000</v>
+      </c>
+      <c r="J27" s="3" t="n">
+        <v>659</v>
+      </c>
+      <c r="K27" t="n">
+        <v>1.14</v>
+      </c>
+      <c r="L27" t="n">
+        <v>22</v>
+      </c>
+      <c r="M27" t="inlineStr">
+        <is>
+          <t>match_type=ppc|organic|section-sponsored-video; score=81.23</t>
+        </is>
+      </c>
+      <c r="N27" s="3" t="n">
+        <v>30048</v>
+      </c>
+      <c r="O27" s="3" t="n">
+        <v>943</v>
+      </c>
+      <c r="P27" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q27" s="2" t="n">
+        <v>10938.8</v>
+      </c>
+      <c r="R27" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S27" s="4" t="n">
+        <v>0.0025591810620601</v>
+      </c>
+      <c r="T27" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="U27" t="n">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>full size bed sheets</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>B00NLLUMOE, B00NQDGAP2, B00O35DAL4, B016P42ARU, B0822X1VP7</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="n">
+        <v>38354</v>
+      </c>
+      <c r="D28" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="E28" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="F28" t="n">
+        <v>70.83504000000001</v>
+      </c>
+      <c r="G28" t="n">
+        <v>3835.4</v>
+      </c>
+      <c r="H28" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="I28" s="3" t="n">
+        <v>10000</v>
+      </c>
+      <c r="J28" s="3" t="n">
+        <v>567</v>
+      </c>
+      <c r="K28" t="n">
+        <v>1.52</v>
+      </c>
+      <c r="L28" t="n">
+        <v>15</v>
+      </c>
+      <c r="M28" t="inlineStr">
+        <is>
+          <t>match_type=organic|sponsored|section-sponsored-video|section-sponsored-brand-header; score=81.94</t>
+        </is>
+      </c>
+      <c r="N28" s="3" t="n">
+        <v>20399</v>
+      </c>
+      <c r="O28" s="3" t="n">
+        <v>464</v>
+      </c>
+      <c r="P28" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q28" s="2" t="n">
+        <v>6992.48</v>
+      </c>
+      <c r="R28" s="2" t="n">
+        <v>107.91</v>
+      </c>
+      <c r="S28" s="4" t="n">
+        <v>0.0058500265910299</v>
+      </c>
+      <c r="T28" s="4" t="n">
+        <v>0.0909090909090909</v>
+      </c>
+      <c r="U28" t="n">
+        <v>30.7</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>bedding</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>B00NLLUMOE, B00NQDGAP2, B00O35DAL4, B016P42ARU, B0822X1VP7</t>
+        </is>
+      </c>
+      <c r="C29" s="3" t="n">
+        <v>69727</v>
+      </c>
+      <c r="D29" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="E29" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="F29" t="n">
+        <v>119.09175</v>
+      </c>
+      <c r="G29" t="n">
+        <v>697.27</v>
+      </c>
+      <c r="H29" s="3" t="n">
+        <v>37</v>
+      </c>
+      <c r="I29" s="3" t="n">
+        <v>100000</v>
+      </c>
+      <c r="J29" s="3" t="n">
+        <v>328</v>
+      </c>
+      <c r="K29" t="n">
+        <v>0.99</v>
+      </c>
+      <c r="L29" t="n">
+        <v>69</v>
+      </c>
+      <c r="M29" t="inlineStr">
+        <is>
+          <t>match_type=ppc|organic|sponsored|section-sponsored-video; score=81.38</t>
+        </is>
+      </c>
+      <c r="U29" t="n">
+        <v>19.2</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>bedsure king comforter set, beige soft prewashed bedding for all seasons, 3 pieces gentlesoft™ bed s</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>B00NLLUMOE, B00NQDGAP2, B00O35DAL4, B016P42ARU, B0822X1VP7</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="n">
+        <v>29186</v>
+      </c>
+      <c r="D30" s="3" t="n">
+        <v>160</v>
+      </c>
+      <c r="E30" s="3" t="n">
+        <v>3</v>
+      </c>
+      <c r="F30" t="n">
+        <v>58.96134000000001</v>
+      </c>
+      <c r="G30" t="n">
+        <v>116278.8844621514</v>
+      </c>
+      <c r="H30" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" s="3" t="n">
+        <v>251</v>
+      </c>
+      <c r="J30" s="3" t="n">
+        <v>220</v>
+      </c>
+      <c r="K30" t="n">
+        <v>1.47</v>
+      </c>
+      <c r="L30" t="n">
+        <v>128</v>
+      </c>
+      <c r="M30" t="inlineStr">
+        <is>
+          <t>match_type=organic|sponsored; score=83.44</t>
+        </is>
+      </c>
+      <c r="U30" t="n">
+        <v>39.9</v>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:U30"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:Q101"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -57298,10 +59345,10 @@
       <c r="O2" t="n">
         <v>365</v>
       </c>
-      <c r="P2" t="n">
+      <c r="P2" s="4" t="n">
         <v>0.008752158066372501</v>
       </c>
-      <c r="Q2" t="n">
+      <c r="Q2" s="4" t="n">
         <v>0.1205479452054794</v>
       </c>
     </row>
@@ -57355,10 +59402,10 @@
       <c r="O3" t="n">
         <v>156</v>
       </c>
-      <c r="P3" t="n">
+      <c r="P3" s="4" t="n">
         <v>0.0063780203606034</v>
       </c>
-      <c r="Q3" t="n">
+      <c r="Q3" s="4" t="n">
         <v>0.1217948717948717</v>
       </c>
     </row>
@@ -57412,10 +59459,10 @@
       <c r="O4" t="n">
         <v>220</v>
       </c>
-      <c r="P4" t="n">
+      <c r="P4" s="4" t="n">
         <v>0.0077065891337093</v>
       </c>
-      <c r="Q4" t="n">
+      <c r="Q4" s="4" t="n">
         <v>0.1136363636363636</v>
       </c>
     </row>
@@ -57469,10 +59516,10 @@
       <c r="O5" t="n">
         <v>50</v>
       </c>
-      <c r="P5" t="n">
+      <c r="P5" s="4" t="n">
         <v>0.004069672798307</v>
       </c>
-      <c r="Q5" t="n">
+      <c r="Q5" s="4" t="n">
         <v>0.1</v>
       </c>
     </row>
@@ -57526,10 +59573,10 @@
       <c r="O6" t="n">
         <v>88</v>
       </c>
-      <c r="P6" t="n">
+      <c r="P6" s="4" t="n">
         <v>0.0064388673446989</v>
       </c>
-      <c r="Q6" t="n">
+      <c r="Q6" s="4" t="n">
         <v>0.1477272727272727</v>
       </c>
     </row>
@@ -57583,10 +59630,10 @@
       <c r="O7" t="n">
         <v>273</v>
       </c>
-      <c r="P7" t="n">
+      <c r="P7" s="4" t="n">
         <v>0.0148055751396496</v>
       </c>
-      <c r="Q7" t="n">
+      <c r="Q7" s="4" t="n">
         <v>0.1355311355311355</v>
       </c>
     </row>
@@ -57640,10 +59687,10 @@
       <c r="O8" t="n">
         <v>93</v>
       </c>
-      <c r="P8" t="n">
+      <c r="P8" s="4" t="n">
         <v>0.0071302614429195</v>
       </c>
-      <c r="Q8" t="n">
+      <c r="Q8" s="4" t="n">
         <v>0.06451612903225799</v>
       </c>
     </row>
@@ -57697,10 +59744,10 @@
       <c r="O9" t="n">
         <v>22</v>
       </c>
-      <c r="P9" t="n">
+      <c r="P9" s="4" t="n">
         <v>0.0040710584752035</v>
       </c>
-      <c r="Q9" t="n">
+      <c r="Q9" s="4" t="n">
         <v>0.0909090909090909</v>
       </c>
     </row>
@@ -57754,10 +59801,10 @@
       <c r="O10" t="n">
         <v>3</v>
       </c>
-      <c r="P10" t="n">
+      <c r="P10" s="4" t="n">
         <v>0.0013428827215756</v>
       </c>
-      <c r="Q10" t="n">
+      <c r="Q10" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -57811,10 +59858,10 @@
       <c r="O11" t="n">
         <v>231</v>
       </c>
-      <c r="P11" t="n">
+      <c r="P11" s="4" t="n">
         <v>0.0100882173115555</v>
       </c>
-      <c r="Q11" t="n">
+      <c r="Q11" s="4" t="n">
         <v>0.0735930735930736</v>
       </c>
     </row>
@@ -57868,10 +59915,10 @@
       <c r="O12" t="n">
         <v>33</v>
       </c>
-      <c r="P12" t="n">
+      <c r="P12" s="4" t="n">
         <v>0.0092931568572233</v>
       </c>
-      <c r="Q12" t="n">
+      <c r="Q12" s="4" t="n">
         <v>0.0303030303030303</v>
       </c>
     </row>
@@ -57925,10 +59972,10 @@
       <c r="O13" t="n">
         <v>23</v>
       </c>
-      <c r="P13" t="n">
+      <c r="P13" s="4" t="n">
         <v>0.0034425984134111</v>
       </c>
-      <c r="Q13" t="n">
+      <c r="Q13" s="4" t="n">
         <v>0.1304347826086956</v>
       </c>
     </row>
@@ -57982,10 +60029,10 @@
       <c r="O14" t="n">
         <v>49</v>
       </c>
-      <c r="P14" t="n">
+      <c r="P14" s="4" t="n">
         <v>0.005789224952741</v>
       </c>
-      <c r="Q14" t="n">
+      <c r="Q14" s="4" t="n">
         <v>0.0612244897959183</v>
       </c>
     </row>
@@ -58039,10 +60086,10 @@
       <c r="O15" t="n">
         <v>499</v>
       </c>
-      <c r="P15" t="n">
+      <c r="P15" s="4" t="n">
         <v>0.009040673974091799</v>
       </c>
-      <c r="Q15" t="n">
+      <c r="Q15" s="4" t="n">
         <v>0.0360721442885771</v>
       </c>
     </row>
@@ -58096,10 +60143,10 @@
       <c r="O16" t="n">
         <v>8</v>
       </c>
-      <c r="P16" t="n">
+      <c r="P16" s="4" t="n">
         <v>0.0025591810620601</v>
       </c>
-      <c r="Q16" t="n">
+      <c r="Q16" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -58153,10 +60200,10 @@
       <c r="O17" t="n">
         <v>10</v>
       </c>
-      <c r="P17" t="n">
+      <c r="P17" s="4" t="n">
         <v>0.0152439024390243</v>
       </c>
-      <c r="Q17" t="n">
+      <c r="Q17" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -58210,10 +60257,10 @@
       <c r="O18" t="n">
         <v>29</v>
       </c>
-      <c r="P18" t="n">
+      <c r="P18" s="4" t="n">
         <v>0.0059401884473576</v>
       </c>
-      <c r="Q18" t="n">
+      <c r="Q18" s="4" t="n">
         <v>0.1724137931034483</v>
       </c>
     </row>
@@ -58267,10 +60314,10 @@
       <c r="O19" t="n">
         <v>157</v>
       </c>
-      <c r="P19" t="n">
+      <c r="P19" s="4" t="n">
         <v>0.0049378833149866</v>
       </c>
-      <c r="Q19" t="n">
+      <c r="Q19" s="4" t="n">
         <v>0.0445859872611464</v>
       </c>
     </row>
@@ -58324,10 +60371,10 @@
       <c r="O20" t="n">
         <v>62</v>
       </c>
-      <c r="P20" t="n">
+      <c r="P20" s="4" t="n">
         <v>0.0094584286803966</v>
       </c>
-      <c r="Q20" t="n">
+      <c r="Q20" s="4" t="n">
         <v>0.1129032258064516</v>
       </c>
     </row>
@@ -58381,10 +60428,10 @@
       <c r="O21" t="n">
         <v>47</v>
       </c>
-      <c r="P21" t="n">
+      <c r="P21" s="4" t="n">
         <v>0.007078313253012</v>
       </c>
-      <c r="Q21" t="n">
+      <c r="Q21" s="4" t="n">
         <v>0.1489361702127659</v>
       </c>
     </row>
@@ -58438,10 +60485,10 @@
       <c r="O22" t="n">
         <v>14</v>
       </c>
-      <c r="P22" t="n">
+      <c r="P22" s="4" t="n">
         <v>0.0135004821600771</v>
       </c>
-      <c r="Q22" t="n">
+      <c r="Q22" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -58495,10 +60542,10 @@
       <c r="O23" t="n">
         <v>41</v>
       </c>
-      <c r="P23" t="n">
+      <c r="P23" s="4" t="n">
         <v>0.009246729815065399</v>
       </c>
-      <c r="Q23" t="n">
+      <c r="Q23" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -58552,10 +60599,10 @@
       <c r="O24" t="n">
         <v>55</v>
       </c>
-      <c r="P24" t="n">
+      <c r="P24" s="4" t="n">
         <v>0.008353584447144499</v>
       </c>
-      <c r="Q24" t="n">
+      <c r="Q24" s="4" t="n">
         <v>0.109090909090909</v>
       </c>
     </row>
@@ -58609,10 +60656,10 @@
       <c r="O25" t="n">
         <v>20</v>
       </c>
-      <c r="P25" t="n">
+      <c r="P25" s="4" t="n">
         <v>0.0137268359643102</v>
       </c>
-      <c r="Q25" t="n">
+      <c r="Q25" s="4" t="n">
         <v>0.05</v>
       </c>
     </row>
@@ -58666,10 +60713,10 @@
       <c r="O26" t="n">
         <v>33</v>
       </c>
-      <c r="P26" t="n">
+      <c r="P26" s="4" t="n">
         <v>0.0058500265910299</v>
       </c>
-      <c r="Q26" t="n">
+      <c r="Q26" s="4" t="n">
         <v>0.0909090909090909</v>
       </c>
     </row>
@@ -58723,10 +60770,10 @@
       <c r="O27" t="n">
         <v>17</v>
       </c>
-      <c r="P27" t="n">
+      <c r="P27" s="4" t="n">
         <v>0.0166994106090373</v>
       </c>
-      <c r="Q27" t="n">
+      <c r="Q27" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -58780,10 +60827,10 @@
       <c r="O28" t="n">
         <v>5</v>
       </c>
-      <c r="P28" t="n">
+      <c r="P28" s="4" t="n">
         <v>0.0047846889952153</v>
       </c>
-      <c r="Q28" t="n">
+      <c r="Q28" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -58834,10 +60881,10 @@
       <c r="O29" t="n">
         <v>5</v>
       </c>
-      <c r="P29" t="n">
+      <c r="P29" s="4" t="n">
         <v>0.0279329608938547</v>
       </c>
-      <c r="Q29" t="n">
+      <c r="Q29" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -58891,10 +60938,10 @@
       <c r="O30" t="n">
         <v>57</v>
       </c>
-      <c r="P30" t="n">
+      <c r="P30" s="4" t="n">
         <v>0.0136887608069164</v>
       </c>
-      <c r="Q30" t="n">
+      <c r="Q30" s="4" t="n">
         <v>0.0526315789473684</v>
       </c>
     </row>
@@ -58948,10 +60995,10 @@
       <c r="O31" t="n">
         <v>9</v>
       </c>
-      <c r="P31" t="n">
+      <c r="P31" s="4" t="n">
         <v>0.0036555645816409</v>
       </c>
-      <c r="Q31" t="n">
+      <c r="Q31" s="4" t="n">
         <v>0.3333333333333333</v>
       </c>
     </row>
@@ -59005,10 +61052,10 @@
       <c r="O32" t="n">
         <v>53</v>
       </c>
-      <c r="P32" t="n">
+      <c r="P32" s="4" t="n">
         <v>0.0122685185185185</v>
       </c>
-      <c r="Q32" t="n">
+      <c r="Q32" s="4" t="n">
         <v>0.2830188679245283</v>
       </c>
     </row>
@@ -59062,7 +61109,7 @@
       <c r="O33" t="n">
         <v>0</v>
       </c>
-      <c r="P33" t="n">
+      <c r="P33" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -59116,10 +61163,10 @@
       <c r="O34" t="n">
         <v>65</v>
       </c>
-      <c r="P34" t="n">
+      <c r="P34" s="4" t="n">
         <v>0.009148486980999199</v>
       </c>
-      <c r="Q34" t="n">
+      <c r="Q34" s="4" t="n">
         <v>0.0769230769230769</v>
       </c>
     </row>
@@ -59173,10 +61220,10 @@
       <c r="O35" t="n">
         <v>6</v>
       </c>
-      <c r="P35" t="n">
+      <c r="P35" s="4" t="n">
         <v>0.003584229390681</v>
       </c>
-      <c r="Q35" t="n">
+      <c r="Q35" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -59230,10 +61277,10 @@
       <c r="O36" t="n">
         <v>8</v>
       </c>
-      <c r="P36" t="n">
+      <c r="P36" s="4" t="n">
         <v>0.0068728522336769</v>
       </c>
-      <c r="Q36" t="n">
+      <c r="Q36" s="4" t="n">
         <v>0.125</v>
       </c>
     </row>
@@ -59287,10 +61334,10 @@
       <c r="O37" t="n">
         <v>13</v>
       </c>
-      <c r="P37" t="n">
+      <c r="P37" s="4" t="n">
         <v>0.0102120974076983</v>
       </c>
-      <c r="Q37" t="n">
+      <c r="Q37" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -59344,10 +61391,10 @@
       <c r="O38" t="n">
         <v>6</v>
       </c>
-      <c r="P38" t="n">
+      <c r="P38" s="4" t="n">
         <v>0.0066371681415929</v>
       </c>
-      <c r="Q38" t="n">
+      <c r="Q38" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -59401,10 +61448,10 @@
       <c r="O39" t="n">
         <v>11</v>
       </c>
-      <c r="P39" t="n">
+      <c r="P39" s="4" t="n">
         <v>0.006979695431472</v>
       </c>
-      <c r="Q39" t="n">
+      <c r="Q39" s="4" t="n">
         <v>0.1818181818181818</v>
       </c>
     </row>
@@ -59458,10 +61505,10 @@
       <c r="O40" t="n">
         <v>23</v>
       </c>
-      <c r="P40" t="n">
+      <c r="P40" s="4" t="n">
         <v>0.0100788781770376</v>
       </c>
-      <c r="Q40" t="n">
+      <c r="Q40" s="4" t="n">
         <v>0.0434782608695652</v>
       </c>
     </row>
@@ -59515,10 +61562,10 @@
       <c r="O41" t="n">
         <v>11</v>
       </c>
-      <c r="P41" t="n">
+      <c r="P41" s="4" t="n">
         <v>0.0055837563451776</v>
       </c>
-      <c r="Q41" t="n">
+      <c r="Q41" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -59572,10 +61619,10 @@
       <c r="O42" t="n">
         <v>2</v>
       </c>
-      <c r="P42" t="n">
+      <c r="P42" s="4" t="n">
         <v>0.0049504950495049</v>
       </c>
-      <c r="Q42" t="n">
+      <c r="Q42" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -59629,10 +61676,10 @@
       <c r="O43" t="n">
         <v>37</v>
       </c>
-      <c r="P43" t="n">
+      <c r="P43" s="4" t="n">
         <v>0.0073093638877913</v>
       </c>
-      <c r="Q43" t="n">
+      <c r="Q43" s="4" t="n">
         <v>0.1351351351351351</v>
       </c>
     </row>
@@ -59686,10 +61733,10 @@
       <c r="O44" t="n">
         <v>28</v>
       </c>
-      <c r="P44" t="n">
+      <c r="P44" s="4" t="n">
         <v>0.0052307117504203</v>
       </c>
-      <c r="Q44" t="n">
+      <c r="Q44" s="4" t="n">
         <v>0.0357142857142857</v>
       </c>
     </row>
@@ -59743,10 +61790,10 @@
       <c r="O45" t="n">
         <v>9</v>
       </c>
-      <c r="P45" t="n">
+      <c r="P45" s="4" t="n">
         <v>0.01931330472103</v>
       </c>
-      <c r="Q45" t="n">
+      <c r="Q45" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -59800,10 +61847,10 @@
       <c r="O46" t="n">
         <v>36</v>
       </c>
-      <c r="P46" t="n">
+      <c r="P46" s="4" t="n">
         <v>0.0071756029499701</v>
       </c>
-      <c r="Q46" t="n">
+      <c r="Q46" s="4" t="n">
         <v>0.0833333333333333</v>
       </c>
     </row>
@@ -59857,10 +61904,10 @@
       <c r="O47" t="n">
         <v>61</v>
       </c>
-      <c r="P47" t="n">
+      <c r="P47" s="4" t="n">
         <v>0.0211585154353104</v>
       </c>
-      <c r="Q47" t="n">
+      <c r="Q47" s="4" t="n">
         <v>0.2459016393442623</v>
       </c>
     </row>
@@ -59914,10 +61961,10 @@
       <c r="O48" t="n">
         <v>7</v>
       </c>
-      <c r="P48" t="n">
+      <c r="P48" s="4" t="n">
         <v>0.0036726128016789</v>
       </c>
-      <c r="Q48" t="n">
+      <c r="Q48" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -59971,10 +62018,10 @@
       <c r="O49" t="n">
         <v>2</v>
       </c>
-      <c r="P49" t="n">
+      <c r="P49" s="4" t="n">
         <v>0.0042372881355932</v>
       </c>
-      <c r="Q49" t="n">
+      <c r="Q49" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -60028,10 +62075,10 @@
       <c r="O50" t="n">
         <v>25</v>
       </c>
-      <c r="P50" t="n">
+      <c r="P50" s="4" t="n">
         <v>0.0073035349108968</v>
       </c>
-      <c r="Q50" t="n">
+      <c r="Q50" s="4" t="n">
         <v>0.08</v>
       </c>
     </row>
@@ -60085,10 +62132,10 @@
       <c r="O51" t="n">
         <v>17</v>
       </c>
-      <c r="P51" t="n">
+      <c r="P51" s="4" t="n">
         <v>0.0043125317097919</v>
       </c>
-      <c r="Q51" t="n">
+      <c r="Q51" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -60142,10 +62189,10 @@
       <c r="O52" t="n">
         <v>68</v>
       </c>
-      <c r="P52" t="n">
+      <c r="P52" s="4" t="n">
         <v>0.0060535920947209</v>
       </c>
-      <c r="Q52" t="n">
+      <c r="Q52" s="4" t="n">
         <v>0.088235294117647</v>
       </c>
     </row>
@@ -60199,10 +62246,10 @@
       <c r="O53" t="n">
         <v>19</v>
       </c>
-      <c r="P53" t="n">
+      <c r="P53" s="4" t="n">
         <v>0.0044496487119437</v>
       </c>
-      <c r="Q53" t="n">
+      <c r="Q53" s="4" t="n">
         <v>0.0526315789473684</v>
       </c>
     </row>
@@ -60256,10 +62303,10 @@
       <c r="O54" t="n">
         <v>8</v>
       </c>
-      <c r="P54" t="n">
+      <c r="P54" s="4" t="n">
         <v>0.0073732718894009</v>
       </c>
-      <c r="Q54" t="n">
+      <c r="Q54" s="4" t="n">
         <v>0.125</v>
       </c>
     </row>
@@ -60313,10 +62360,10 @@
       <c r="O55" t="n">
         <v>28</v>
       </c>
-      <c r="P55" t="n">
+      <c r="P55" s="4" t="n">
         <v>0.0050152247895396</v>
       </c>
-      <c r="Q55" t="n">
+      <c r="Q55" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -60367,10 +62414,10 @@
       <c r="O56" t="n">
         <v>4</v>
       </c>
-      <c r="P56" t="n">
+      <c r="P56" s="4" t="n">
         <v>0.0164609053497942</v>
       </c>
-      <c r="Q56" t="n">
+      <c r="Q56" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -60424,10 +62471,10 @@
       <c r="O57" t="n">
         <v>26</v>
       </c>
-      <c r="P57" t="n">
+      <c r="P57" s="4" t="n">
         <v>0.0193885160328113</v>
       </c>
-      <c r="Q57" t="n">
+      <c r="Q57" s="4" t="n">
         <v>0.3076923076923077</v>
       </c>
     </row>
@@ -60478,10 +62525,10 @@
       <c r="O58" t="n">
         <v>1</v>
       </c>
-      <c r="P58" t="n">
+      <c r="P58" s="4" t="n">
         <v>0.0035714285714285</v>
       </c>
-      <c r="Q58" t="n">
+      <c r="Q58" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -60535,7 +62582,7 @@
       <c r="O59" t="n">
         <v>0</v>
       </c>
-      <c r="P59" t="n">
+      <c r="P59" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -60589,10 +62636,10 @@
       <c r="O60" t="n">
         <v>2</v>
       </c>
-      <c r="P60" t="n">
+      <c r="P60" s="4" t="n">
         <v>0.0023041474654377</v>
       </c>
-      <c r="Q60" t="n">
+      <c r="Q60" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -60646,10 +62693,10 @@
       <c r="O61" t="n">
         <v>40</v>
       </c>
-      <c r="P61" t="n">
+      <c r="P61" s="4" t="n">
         <v>0.0269541778975741</v>
       </c>
-      <c r="Q61" t="n">
+      <c r="Q61" s="4" t="n">
         <v>0.175</v>
       </c>
     </row>
@@ -60703,7 +62750,7 @@
       <c r="O62" t="n">
         <v>0</v>
       </c>
-      <c r="P62" t="n">
+      <c r="P62" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -60757,10 +62804,10 @@
       <c r="O63" t="n">
         <v>5</v>
       </c>
-      <c r="P63" t="n">
+      <c r="P63" s="4" t="n">
         <v>0.0072886297376093</v>
       </c>
-      <c r="Q63" t="n">
+      <c r="Q63" s="4" t="n">
         <v>0.2</v>
       </c>
     </row>
@@ -60814,10 +62861,10 @@
       <c r="O64" t="n">
         <v>9</v>
       </c>
-      <c r="P64" t="n">
+      <c r="P64" s="4" t="n">
         <v>0.009933774834437</v>
       </c>
-      <c r="Q64" t="n">
+      <c r="Q64" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -60871,10 +62918,10 @@
       <c r="O65" t="n">
         <v>4</v>
       </c>
-      <c r="P65" t="n">
+      <c r="P65" s="4" t="n">
         <v>0.0028653295128939</v>
       </c>
-      <c r="Q65" t="n">
+      <c r="Q65" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -60928,10 +62975,10 @@
       <c r="O66" t="n">
         <v>30</v>
       </c>
-      <c r="P66" t="n">
+      <c r="P66" s="4" t="n">
         <v>0.0041823504809703</v>
       </c>
-      <c r="Q66" t="n">
+      <c r="Q66" s="4" t="n">
         <v>0.0333333333333333</v>
       </c>
     </row>
@@ -60985,10 +63032,10 @@
       <c r="O67" t="n">
         <v>8</v>
       </c>
-      <c r="P67" t="n">
+      <c r="P67" s="4" t="n">
         <v>0.0098643649815043</v>
       </c>
-      <c r="Q67" t="n">
+      <c r="Q67" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -61042,10 +63089,10 @@
       <c r="O68" t="n">
         <v>12</v>
       </c>
-      <c r="P68" t="n">
+      <c r="P68" s="4" t="n">
         <v>0.0073982737361282</v>
       </c>
-      <c r="Q68" t="n">
+      <c r="Q68" s="4" t="n">
         <v>0.0833333333333333</v>
       </c>
     </row>
@@ -61096,10 +63143,10 @@
       <c r="O69" t="n">
         <v>1</v>
       </c>
-      <c r="P69" t="n">
+      <c r="P69" s="4" t="n">
         <v>0.002906976744186</v>
       </c>
-      <c r="Q69" t="n">
+      <c r="Q69" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -61153,10 +63200,10 @@
       <c r="O70" t="n">
         <v>11</v>
       </c>
-      <c r="P70" t="n">
+      <c r="P70" s="4" t="n">
         <v>0.0098302055406613</v>
       </c>
-      <c r="Q70" t="n">
+      <c r="Q70" s="4" t="n">
         <v>0.1818181818181818</v>
       </c>
     </row>
@@ -61210,10 +63257,10 @@
       <c r="O71" t="n">
         <v>16</v>
       </c>
-      <c r="P71" t="n">
+      <c r="P71" s="4" t="n">
         <v>0.0126182965299684</v>
       </c>
-      <c r="Q71" t="n">
+      <c r="Q71" s="4" t="n">
         <v>0.3125</v>
       </c>
     </row>
@@ -61267,10 +63314,10 @@
       <c r="O72" t="n">
         <v>2</v>
       </c>
-      <c r="P72" t="n">
+      <c r="P72" s="4" t="n">
         <v>0.0037105751391465</v>
       </c>
-      <c r="Q72" t="n">
+      <c r="Q72" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -61324,10 +63371,10 @@
       <c r="O73" t="n">
         <v>5</v>
       </c>
-      <c r="P73" t="n">
+      <c r="P73" s="4" t="n">
         <v>0.0141242937853107</v>
       </c>
-      <c r="Q73" t="n">
+      <c r="Q73" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -61381,10 +63428,10 @@
       <c r="O74" t="n">
         <v>2</v>
       </c>
-      <c r="P74" t="n">
+      <c r="P74" s="4" t="n">
         <v>0.0030257186081694</v>
       </c>
-      <c r="Q74" t="n">
+      <c r="Q74" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -61438,10 +63485,10 @@
       <c r="O75" t="n">
         <v>4</v>
       </c>
-      <c r="P75" t="n">
+      <c r="P75" s="4" t="n">
         <v>0.0074074074074074</v>
       </c>
-      <c r="Q75" t="n">
+      <c r="Q75" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -61495,10 +63542,10 @@
       <c r="O76" t="n">
         <v>2</v>
       </c>
-      <c r="P76" t="n">
+      <c r="P76" s="4" t="n">
         <v>0.0020304568527918</v>
       </c>
-      <c r="Q76" t="n">
+      <c r="Q76" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -61552,10 +63599,10 @@
       <c r="O77" t="n">
         <v>1</v>
       </c>
-      <c r="P77" t="n">
+      <c r="P77" s="4" t="n">
         <v>0.0034602076124567</v>
       </c>
-      <c r="Q77" t="n">
+      <c r="Q77" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -61606,10 +63653,10 @@
       <c r="O78" t="n">
         <v>1</v>
       </c>
-      <c r="P78" t="n">
+      <c r="P78" s="4" t="n">
         <v>0.0032362459546925</v>
       </c>
-      <c r="Q78" t="n">
+      <c r="Q78" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -61663,10 +63710,10 @@
       <c r="O79" t="n">
         <v>6</v>
       </c>
-      <c r="P79" t="n">
+      <c r="P79" s="4" t="n">
         <v>0.0027790643816581</v>
       </c>
-      <c r="Q79" t="n">
+      <c r="Q79" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -61720,7 +63767,7 @@
       <c r="O80" t="n">
         <v>0</v>
       </c>
-      <c r="P80" t="n">
+      <c r="P80" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -61774,10 +63821,10 @@
       <c r="O81" t="n">
         <v>1</v>
       </c>
-      <c r="P81" t="n">
+      <c r="P81" s="4" t="n">
         <v>0.002710027100271</v>
       </c>
-      <c r="Q81" t="n">
+      <c r="Q81" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -61831,7 +63878,7 @@
       <c r="O82" t="n">
         <v>0</v>
       </c>
-      <c r="P82" t="n">
+      <c r="P82" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -61885,10 +63932,10 @@
       <c r="O83" t="n">
         <v>3</v>
       </c>
-      <c r="P83" t="n">
+      <c r="P83" s="4" t="n">
         <v>0.008064516129032201</v>
       </c>
-      <c r="Q83" t="n">
+      <c r="Q83" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -61939,10 +63986,10 @@
       <c r="O84" t="n">
         <v>3</v>
       </c>
-      <c r="P84" t="n">
+      <c r="P84" s="4" t="n">
         <v>0.0138888888888888</v>
       </c>
-      <c r="Q84" t="n">
+      <c r="Q84" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -61993,7 +64040,7 @@
       <c r="O85" t="n">
         <v>0</v>
       </c>
-      <c r="P85" t="n">
+      <c r="P85" s="4" t="n">
         <v>0</v>
       </c>
     </row>
@@ -62047,10 +64094,10 @@
       <c r="O86" t="n">
         <v>7</v>
       </c>
-      <c r="P86" t="n">
+      <c r="P86" s="4" t="n">
         <v>0.0136452241715399</v>
       </c>
-      <c r="Q86" t="n">
+      <c r="Q86" s="4" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>